<commit_message>
update dp pract 04e77950704d12c2331a8a3b76e099452e25ce00
</commit_message>
<xml_diff>
--- a/nr-change-vs-address-disctrict/ig/StructureDefinition-as-dp-practitioner.xlsx
+++ b/nr-change-vs-address-disctrict/ig/StructureDefinition-as-dp-practitioner.xlsx
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2025-02-06T17:38:45+00:00</t>
+    <t>2025-02-11T12:23:43+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -15640,7 +15640,7 @@
         <v>85</v>
       </c>
       <c r="G90" t="s" s="2">
-        <v>102</v>
+        <v>86</v>
       </c>
       <c r="H90" t="s" s="2">
         <v>103</v>

</xml_diff>